<commit_message>
make backend for stories, index & saved
</commit_message>
<xml_diff>
--- a/travel_stories_50_dummy_data.xlsx
+++ b/travel_stories_50_dummy_data.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="76">
   <si>
     <t>Title</t>
   </si>
@@ -247,13 +247,16 @@
   </si>
   <si>
     <t>Image</t>
+  </si>
+  <si>
+    <t>https://img.magnific.com/premium-photo/spring-kullu-valley-himalaya-mountains-himachal-pradesh-india_163782-2284.jpg?semt=ais_hybrid&amp;w=740&amp;q=80</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -270,6 +273,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -307,10 +318,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -318,8 +330,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -660,9 +674,8 @@
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="str">
-        <f>"https://www.sourcesplash.com/i/random?q="&amp;SUBSTITUTE(B2," ","%20")</f>
-        <v>https://www.sourcesplash.com/i/random?q=Manali,%20Himachal%20Pradesh</v>
+      <c r="E2" s="3" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1549,7 +1562,10 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D51"/>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>